<commit_message>
feat(onboarding): seed recurring and rules in sample workbook
</commit_message>
<xml_diff>
--- a/public/sample-onboarding-import.xlsx
+++ b/public/sample-onboarding-import.xlsx
@@ -7,6 +7,8 @@
     <sheet name="Budgets" sheetId="2" r:id="rId2"/>
     <sheet name="Goals" sheetId="3" r:id="rId3"/>
     <sheet name="Transactions" sheetId="4" r:id="rId4"/>
+    <sheet name="Recurring" sheetId="5" r:id="rId5"/>
+    <sheet name="Rules" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -5665,4 +5667,331 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J135"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>title</v>
+      </c>
+      <c r="B1" t="str">
+        <v>type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="D1" t="str">
+        <v>category</v>
+      </c>
+      <c r="E1" t="str">
+        <v>accountName</v>
+      </c>
+      <c r="F1" t="str">
+        <v>frequency</v>
+      </c>
+      <c r="G1" t="str">
+        <v>startDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>endDate</v>
+      </c>
+      <c r="I1" t="str">
+        <v>nextRunDate</v>
+      </c>
+      <c r="J1" t="str">
+        <v>autoCreateTransaction</v>
+      </c>
+      <c r="K1" t="str">
+        <v>isPaused</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Monthly Salary</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Income</v>
+      </c>
+      <c r="C2">
+        <v>72000</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Horizon Checking</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-10-01</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-03-01</v>
+      </c>
+      <c r="J2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="K2" t="str">
+        <v>FALSE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Apartment Rent</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="C3">
+        <v>19500</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Horizon Checking</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-10-03</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-03-03</v>
+      </c>
+      <c r="J3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="K3" t="str">
+        <v>FALSE</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Subscription Stack</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="C4">
+        <v>1198</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Entertainment</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Atlas Credit Card</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-10-13</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-03-13</v>
+      </c>
+      <c r="J4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="K4" t="str">
+        <v>FALSE</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Emergency Fund Transfer</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="C5">
+        <v>9500</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Others</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Horizon Checking</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Monthly</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2025-10-08</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-03-08</v>
+      </c>
+      <c r="J5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="K5" t="str">
+        <v>FALSE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>conditionField</v>
+      </c>
+      <c r="C1" t="str">
+        <v>conditionOperator</v>
+      </c>
+      <c r="D1" t="str">
+        <v>conditionValue</v>
+      </c>
+      <c r="E1" t="str">
+        <v>actionType</v>
+      </c>
+      <c r="F1" t="str">
+        <v>actionValue</v>
+      </c>
+      <c r="G1" t="str">
+        <v>priority</v>
+      </c>
+      <c r="H1" t="str">
+        <v>isActive</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Auto-tag food delivery</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Merchant</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Contains</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Swiggy</v>
+      </c>
+      <c r="E2" t="str">
+        <v>AddTag</v>
+      </c>
+      <c r="F2" t="str">
+        <v>food-delivery</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Map Fresh Basket to Groceries</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Merchant</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Contains</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Fresh Basket</v>
+      </c>
+      <c r="E3" t="str">
+        <v>SetCategory</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Flag large travel charges</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Category</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Equals</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="E4" t="str">
+        <v>TriggerAlert</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Review large travel expense</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Tag subscriptions</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Merchant</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Contains</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E5" t="str">
+        <v>AddTag</v>
+      </c>
+      <c r="F5" t="str">
+        <v>subscription</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): surface credit card limit tracking
</commit_message>
<xml_diff>
--- a/public/sample-onboarding-import.xlsx
+++ b/public/sample-onboarding-import.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,6 +417,9 @@
       <c r="D1" t="str">
         <v>institutionName</v>
       </c>
+      <c r="E1" t="str">
+        <v>creditLimit</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -459,6 +462,9 @@
       <c r="D4" t="str">
         <v>Axis Bank</v>
       </c>
+      <c r="E4">
+        <v>90000</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -476,7 +482,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(ui): sync legacy onboarding sample workbook
</commit_message>
<xml_diff>
--- a/public/sample-onboarding-import.xlsx
+++ b/public/sample-onboarding-import.xlsx
@@ -418,7 +418,7 @@
         <v>institutionName</v>
       </c>
       <c r="E1" t="str">
-        <v>creditLimit</v>
+        <v>limit</v>
       </c>
     </row>
     <row r="2">
@@ -433,6 +433,9 @@
       </c>
       <c r="D2" t="str">
         <v>HDFC Bank</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -448,6 +451,9 @@
       <c r="D3" t="str">
         <v>ICICI Bank</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -478,6 +484,9 @@
       </c>
       <c r="D5" t="str">
         <v>Wallet</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>